<commit_message>
data builder fix for direct and PCW
</commit_message>
<xml_diff>
--- a/sampleData/New Business.xlsx
+++ b/sampleData/New Business.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijaytomar/AZOnline_Automation/AZOnline/sampleData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B956CCF-E4B9-BB46-BA4C-F32B089475FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFA2CE6-2068-2046-B76C-4486575037CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master_Template" sheetId="1" r:id="rId1"/>
     <sheet name="FlowNB" sheetId="2" r:id="rId2"/>
-    <sheet name="PCW Tool" sheetId="4" r:id="rId3"/>
-    <sheet name="Conventions" sheetId="3" r:id="rId4"/>
+    <sheet name="PCW Tool_New" sheetId="4" r:id="rId3"/>
+    <sheet name="PCW Tool" sheetId="5" r:id="rId4"/>
+    <sheet name="Conventions" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6312" uniqueCount="1106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6354" uniqueCount="1111">
   <si>
     <t>Section</t>
   </si>
@@ -3341,6 +3342,21 @@
   </si>
   <si>
     <t>{"Risk":{  "Proposer": {    "AllowContact": [      {        "Subscription": "ThirdPartyContact",        "Allowed": false      },      {        "Subscription": "ContactConsentForActivity",        "Allowed": true      }    ],    "PersonsOnPolicy": "YourselfOnly",    "VehiclesInHousehold": 1,    "HasHeldInsuranceWithinLastTwoYears": false,    "RegularNamedDriver": false,    "YearsClaimFreeDrivingExperience": "NotSelected",    "PreviousDrivingExperience": "NotSpecified",    "NoClaimsBonus": "FourYears",    "HomeOwner": false,    "HasChildrenUnderSixteen": false,    "PaymentMethod": "Annual",    "ContactDetails": {      "PhoneNumber": "07777 777889",      "CorrespondenceAddress": {        "Postcode": {          "OutwardCode": "TR1",          "InwardCode": "3PE"        },        "HouseNumber": "32",        "Road": "Cornish Crescent",        "Town": "Truro",        "County": "Cornwall"      },      "EmailAddress": "allianz.test.sd+Confused_RegTC010_10_07_25_06@gmail.com",      "OutboundByInsurer": false    },    "MainDriver": true,    "UseOfOtherCars": false,    "LicenceType": "FullUkManual",    "DateLicenceObtained": "2013-09-15",    "DateUKResidentSince": "1981-07-21",    "DVLAMedicalCondition": "NotApplicable",    "OtherCarOwnedInsured": false,    "InsuranceDeclinedOrCancelled": false,    "NonMotoringConvictions": false,    "PassPlus": false,    "OtherVehicleType": "No",    "PrimaryOccupation": {      "EmploymentStatus": "Employed",      "Occupation": "AccountManager",      "BusinessType": "Banking"    },    "Convictions": [      {        "Date": "2020-06-01",        "Points": 3,        "FineAmount": 60.0,        "BanLength": 0,        "AccidentRelated": false,        "DVLACode": "PC20",        "WasBreathalysed": false      },      {        "Date": "2019-08-01",        "Points": 3,        "FineAmount": 60.0,        "BanLength": 0,        "AccidentRelated": false,        "DVLACode": "TS30",        "WasBreathalysed": false      }    ],    "Title": "Miss",    "MaritalStatus": "CommonLaw",    "FirstName": "Anna",    "Surname": "Cole",    "DateOfBirth": "1981-07-21"  },  "Vehicle": {    "AbiCode": "33806101",    "Make": "MINI",    "Model": "COOPER",    "Variant": "01",    "BodyStyle": "ThreeDoorHatchback",    "Doors": 3,    "EngineSize": 1598,    "Year": 2011,    "FuelType": "Petrol",    "Transmission": "Manual",    "Value": 4895,    "Alarm": "AlarmFitted",    "ImmobiliserMake": "ThatchamOneOrTwo",    "TrackerMake": "None",    "RegistrationNumber": "SH11UKA",    "DatePurchased": "2021-01-01",    "DriverSide": "Right",    "RegisteredKeeper": "PolicyHolder",    "LegalOwner": "PolicyHolder",    "ImportType": "NoStandardUkModel",    "Seats": 4,    "Purchased": true,    "OvernightLocation": "Garage",    "DaytimeLocation": "AtHome",    "HasDashCam": false,    "DateFirstRegistered": "2011-05-14",    "PostCodeKept": {      "OutwardCode": "TR1",      "InwardCode": "3PE"    }  },  "CoverUse": {    "ClassOfUse": "SocialOnly",    "ProtectedNoClaimsBonus": "NoProtection",    "CoverType": "Comprehensive",    "TotalAnnualMileage": "UpTo8000",    "BusinessMileage": "None",    "VoluntaryExcess": "Amount350",    "DateCoverRequired": "2023-09-26"  }},"ActivityId" : "07597f23-f9cb-4c91-b938-c034257d401d"}</t>
+  </si>
+  <si>
+    <t>PCW_TC001</t>
+  </si>
+  <si>
+    <t>PCW_TC002</t>
+  </si>
+  <si>
+    <t>PCW Monthly Flow</t>
+  </si>
+  <si>
+    <t>PCW Annual Flow</t>
+  </si>
+  <si>
+    <t>PcwTool</t>
   </si>
 </sst>
 </file>
@@ -28705,6 +28721,177 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8DD7EA-FB71-4249-95D7-B42E92EACA33}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1097</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1108</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>948</v>
+      </c>
+      <c r="D5" t="s">
+        <v>948</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B11" t="s">
+        <v>928</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1099</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>938</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76B13375-6280-0447-A001-5D49208C67B8}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -28788,7 +28975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
tree view change for execution layer
</commit_message>
<xml_diff>
--- a/sampleData/New Business.xlsx
+++ b/sampleData/New Business.xlsx
@@ -8,23 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijaytomar/AZOnline_Automation/AZOnline/sampleData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CFA2CE6-2068-2046-B76C-4486575037CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319CEEB8-D709-FF40-ABC0-2F7F3ED29E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master_Template" sheetId="1" r:id="rId1"/>
     <sheet name="FlowNB" sheetId="2" r:id="rId2"/>
-    <sheet name="PCW Tool_New" sheetId="4" r:id="rId3"/>
-    <sheet name="PCW Tool" sheetId="5" r:id="rId4"/>
-    <sheet name="Conventions" sheetId="3" r:id="rId5"/>
+    <sheet name="PCW Tool" sheetId="5" r:id="rId3"/>
+    <sheet name="Conventions" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6354" uniqueCount="1111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6312" uniqueCount="1106">
   <si>
     <t>Section</t>
   </si>
@@ -3342,21 +3341,6 @@
   </si>
   <si>
     <t>{"Risk":{  "Proposer": {    "AllowContact": [      {        "Subscription": "ThirdPartyContact",        "Allowed": false      },      {        "Subscription": "ContactConsentForActivity",        "Allowed": true      }    ],    "PersonsOnPolicy": "YourselfOnly",    "VehiclesInHousehold": 1,    "HasHeldInsuranceWithinLastTwoYears": false,    "RegularNamedDriver": false,    "YearsClaimFreeDrivingExperience": "NotSelected",    "PreviousDrivingExperience": "NotSpecified",    "NoClaimsBonus": "FourYears",    "HomeOwner": false,    "HasChildrenUnderSixteen": false,    "PaymentMethod": "Annual",    "ContactDetails": {      "PhoneNumber": "07777 777889",      "CorrespondenceAddress": {        "Postcode": {          "OutwardCode": "TR1",          "InwardCode": "3PE"        },        "HouseNumber": "32",        "Road": "Cornish Crescent",        "Town": "Truro",        "County": "Cornwall"      },      "EmailAddress": "allianz.test.sd+Confused_RegTC010_10_07_25_06@gmail.com",      "OutboundByInsurer": false    },    "MainDriver": true,    "UseOfOtherCars": false,    "LicenceType": "FullUkManual",    "DateLicenceObtained": "2013-09-15",    "DateUKResidentSince": "1981-07-21",    "DVLAMedicalCondition": "NotApplicable",    "OtherCarOwnedInsured": false,    "InsuranceDeclinedOrCancelled": false,    "NonMotoringConvictions": false,    "PassPlus": false,    "OtherVehicleType": "No",    "PrimaryOccupation": {      "EmploymentStatus": "Employed",      "Occupation": "AccountManager",      "BusinessType": "Banking"    },    "Convictions": [      {        "Date": "2020-06-01",        "Points": 3,        "FineAmount": 60.0,        "BanLength": 0,        "AccidentRelated": false,        "DVLACode": "PC20",        "WasBreathalysed": false      },      {        "Date": "2019-08-01",        "Points": 3,        "FineAmount": 60.0,        "BanLength": 0,        "AccidentRelated": false,        "DVLACode": "TS30",        "WasBreathalysed": false      }    ],    "Title": "Miss",    "MaritalStatus": "CommonLaw",    "FirstName": "Anna",    "Surname": "Cole",    "DateOfBirth": "1981-07-21"  },  "Vehicle": {    "AbiCode": "33806101",    "Make": "MINI",    "Model": "COOPER",    "Variant": "01",    "BodyStyle": "ThreeDoorHatchback",    "Doors": 3,    "EngineSize": 1598,    "Year": 2011,    "FuelType": "Petrol",    "Transmission": "Manual",    "Value": 4895,    "Alarm": "AlarmFitted",    "ImmobiliserMake": "ThatchamOneOrTwo",    "TrackerMake": "None",    "RegistrationNumber": "SH11UKA",    "DatePurchased": "2021-01-01",    "DriverSide": "Right",    "RegisteredKeeper": "PolicyHolder",    "LegalOwner": "PolicyHolder",    "ImportType": "NoStandardUkModel",    "Seats": 4,    "Purchased": true,    "OvernightLocation": "Garage",    "DaytimeLocation": "AtHome",    "HasDashCam": false,    "DateFirstRegistered": "2011-05-14",    "PostCodeKept": {      "OutwardCode": "TR1",      "InwardCode": "3PE"    }  },  "CoverUse": {    "ClassOfUse": "SocialOnly",    "ProtectedNoClaimsBonus": "NoProtection",    "CoverType": "Comprehensive",    "TotalAnnualMileage": "UpTo8000",    "BusinessMileage": "None",    "VoluntaryExcess": "Amount350",    "DateCoverRequired": "2023-09-26"  }},"ActivityId" : "07597f23-f9cb-4c91-b938-c034257d401d"}</t>
-  </si>
-  <si>
-    <t>PCW_TC001</t>
-  </si>
-  <si>
-    <t>PCW_TC002</t>
-  </si>
-  <si>
-    <t>PCW Monthly Flow</t>
-  </si>
-  <si>
-    <t>PCW Annual Flow</t>
-  </si>
-  <si>
-    <t>PcwTool</t>
   </si>
 </sst>
 </file>
@@ -28720,177 +28704,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B8DD7EA-FB71-4249-95D7-B42E92EACA33}">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1097</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>1106</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1107</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>1108</v>
-      </c>
-      <c r="D4" t="s">
-        <v>1109</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
-        <v>948</v>
-      </c>
-      <c r="D5" t="s">
-        <v>948</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1093</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1097</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C8" t="s">
-        <v>1104</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1105</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B9" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1096</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1098</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1101</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B11" t="s">
-        <v>928</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1099</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>1110</v>
-      </c>
-      <c r="B12" t="s">
-        <v>938</v>
-      </c>
-      <c r="D12" t="s">
-        <v>1103</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76B13375-6280-0447-A001-5D49208C67B8}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -28975,7 +28788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>